<commit_message>
Allow postgraduate project groups A1-A50 in student import and fix student email domains
</commit_message>
<xml_diff>
--- a/csv_uploads/student_supervisor_allocation.xlsx
+++ b/csv_uploads/student_supervisor_allocation.xlsx
@@ -1639,7 +1639,7 @@
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>nanatenkorang.opoku@st.gimpa.edu</t>
+          <t>nanatenkorang.opoku@st.gimpa.edu.gh</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>abdul-aziz.adams@st.gimpa.edu</t>
+          <t>abdul-aziz.adams@st.gimpa.edu.gh</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">

</xml_diff>